<commit_message>
2025-10-10 Calibration gui ok
</commit_message>
<xml_diff>
--- a/Firmware/Firmware_Requiremnts.xlsx
+++ b/Firmware/Firmware_Requiremnts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Academic\UOC\Reaserch\LowPowerDataLogger\Firmware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB08B142-BFB5-4920-A8B4-5097BCE58626}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE3E9D3-6D29-498D-B886-723C947FCEA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="52">
   <si>
     <t>Requirement</t>
   </si>
@@ -178,6 +178,9 @@
   </si>
   <si>
     <t xml:space="preserve">                                   Set heartbeat STATUS LED </t>
+  </si>
+  <si>
+    <t>NO</t>
   </si>
 </sst>
 </file>
@@ -948,33 +951,69 @@
       <c r="A63" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B63" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B65" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B66" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B67" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B68" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B69" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>47</v>
       </c>

</xml_diff>